<commit_message>
Halloween songs: 10 clips (echo & dry) cut and on the board
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/songs.xlsx
+++ b/tools/songs.xlsx
@@ -1283,13 +1283,20 @@
       <c r="A35" t="n">
         <v>1</v>
       </c>
-      <c r="B35" s="2" t="n"/>
+      <c r="B35" s="2" t="n">
+        <v>577</v>
+      </c>
       <c r="C35" s="2" t="n"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Thriller</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Michael Jackson - Thriller (Official 4K Video).m4a</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1297,7 +1304,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>to download: Michael Jackson - Thriller</t>
+          <t>start: loudest minute of the short film; listen (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1305,13 +1312,20 @@
       <c r="A36" t="n">
         <v>1</v>
       </c>
-      <c r="B36" s="2" t="n"/>
+      <c r="B36" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="C36" s="2" t="n"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>MonsterMash</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Bobby Pickett - Monster Mash [HD].m4a</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1319,7 +1333,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>to download: Bobby "Boris" Pickett - Monster Mash</t>
+          <t>start: from the top (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1327,13 +1341,20 @@
       <c r="A37" t="n">
         <v>2</v>
       </c>
-      <c r="B37" s="2" t="n"/>
+      <c r="B37" s="2" t="n">
+        <v>177</v>
+      </c>
       <c r="C37" s="2" t="n"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>Ghostbusters</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Ray Parker Jr. - Ghostbusters (Official HD Video).m4a</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1341,7 +1362,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>to download: Ray Parker Jr. - Ghostbusters</t>
+          <t>start: loudest minute (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1349,13 +1370,20 @@
       <c r="A38" t="n">
         <v>2</v>
       </c>
-      <c r="B38" s="2" t="n"/>
+      <c r="B38" s="2" t="n">
+        <v>83</v>
+      </c>
       <c r="C38" s="2" t="n"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>ThisIsHalloween</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\The Citizens of Halloween - This Is Halloween (From Tim Burton's  The Nightmare Before Christmas ).m4a</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1363,7 +1391,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>to download: The Nightmare Before Christmas - This Is Halloween</t>
+          <t>start: loudest minute (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1371,13 +1399,20 @@
       <c r="A39" t="n">
         <v>3</v>
       </c>
-      <c r="B39" s="2" t="n"/>
+      <c r="B39" s="2" t="n">
+        <v>131</v>
+      </c>
       <c r="C39" s="2" t="n"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>TimeWarp</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Let's Do The TIME WARP Again!    The Rocky Horror Picture Show  (4K).m4a</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1385,7 +1420,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>to download: Rocky Horror Picture Show - Time Warp</t>
+          <t>start: loudest minute (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1415,13 +1450,20 @@
       <c r="A41" t="n">
         <v>4</v>
       </c>
-      <c r="B41" s="2" t="n"/>
+      <c r="B41" s="2" t="n">
+        <v>45</v>
+      </c>
       <c r="C41" s="2" t="n"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>SpookyScarySkeletons</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Andrew Gold - Spooky Scary Skeletons (Official Audio).m4a</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1429,7 +1471,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>to download: Andrew Gold - Spooky Scary Skeletons</t>
+          <t>start: loudest minute (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1437,13 +1479,20 @@
       <c r="A42" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="2" t="n"/>
+      <c r="B42" s="2" t="n">
+        <v>71</v>
+      </c>
       <c r="C42" s="2" t="n"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>PurplePeopleEater</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Sheb Wooley  The Purple People Eater  (Official Video).m4a</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1451,7 +1500,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>to download: Sheb Wooley - The Purple People Eater</t>
+          <t>start: loudest minute (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1459,13 +1508,20 @@
       <c r="A43" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="2" t="n"/>
+      <c r="B43" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="C43" s="2" t="n"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>AddamsFamily</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\Vic Mizzy - Main Theme The Addams Family (Official Audio).m4a</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1473,7 +1529,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>to download: Vic Mizzy - The Addams Family Theme</t>
+          <t>start: whole theme (55 s) (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1503,13 +1559,20 @@
       <c r="A45" t="n">
         <v>6</v>
       </c>
-      <c r="B45" s="2" t="n"/>
+      <c r="B45" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="C45" s="2" t="n"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>Toccata</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\J.S. Bach  Toccata and Fugue in D minor BWV 565   Liene Andreta Kalnciema live at Riga Cathedral.m4a</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1517,7 +1580,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>to download: Bach - Toccata and Fugue in D minor (organ)</t>
+          <t>start: the famous opening (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -1525,13 +1588,20 @@
       <c r="A46" t="n">
         <v>6</v>
       </c>
-      <c r="B46" s="2" t="n"/>
+      <c r="B46" s="2" t="n">
+        <v>75</v>
+      </c>
       <c r="C46" s="2" t="n"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>WitchDoctor</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>D:\Muzak\JohnsMusic\halloween\David Seville - Witch Doctor [Remastered].m4a</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>halloween</t>
@@ -1539,7 +1609,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>to download: David Seville - Witch Doctor</t>
+          <t>start: loudest minute (Claude 2026-10-30)</t>
         </is>
       </c>
     </row>

</xml_diff>